<commit_message>
Fix file template fallback, BoE quantity extraction, and Web GUI execution
</commit_message>
<xml_diff>
--- a/output/master_reviewed.xlsx
+++ b/output/master_reviewed.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,11 +543,7 @@
           <t>032-1 CD70 SM 032 Analog output</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="n">
         <v>7.5</v>
       </c>
@@ -578,11 +574,7 @@
           <t>972-0DP30 EasyConn 00 PB plug</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>85366990</t>
-        </is>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>10</v>
       </c>
@@ -613,11 +605,7 @@
           <t>001-1 BAOO CM 001 Pot. distributor</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>85369090</t>
-        </is>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
         <v>10</v>
       </c>
@@ -648,11 +636,7 @@
           <t>001-1BAIO CM 001 pot. distributor</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>85369090</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
       <c r="E7" t="n">
         <v>10</v>
       </c>
@@ -683,7 +667,11 @@
           <t>007-IABOO PM 007 Power module</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>85366990</t>
+        </is>
+      </c>
       <c r="E8" t="n">
         <v>10</v>
       </c>
@@ -714,7 +702,11 @@
           <t>021-1 BFOO SM 021 Digital input</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
       <c r="E9" t="n">
         <v>7.5</v>
       </c>
@@ -1158,11 +1150,7 @@
           <t>314-2AG23 VIPA CPU 314SB DPM</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="n">
         <v>7.5</v>
       </c>
@@ -1386,7 +1374,11 @@
           <t>031-1BD40 SM 031 Analog input</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
       <c r="E33" t="n">
         <v>7.5</v>
       </c>
@@ -1541,11 +1533,7 @@
           <t>032-1 BB40 SM 032 Analog output</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>7.5</v>
       </c>
@@ -1731,7 +1719,11 @@
           <t>H41-71A41-0 smartPanel TP304-SM</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
       <c r="E44" t="n">
         <v>7.5</v>
       </c>
@@ -1762,7 +1754,11 @@
           <t>1-171-71 A 41-0 smartPanel TP307-SM</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
       <c r="E45" t="n">
         <v>7.5</v>
       </c>
@@ -1824,7 +1820,11 @@
           <t>015-CEFPROI CPU 015PN</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
       <c r="E47" t="n">
         <v>7.5</v>
       </c>
@@ -1948,7 +1948,11 @@
           <t>001-1BA20 CM 001 pot. distributor</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>85366990</t>
+        </is>
+      </c>
       <c r="E51" t="n">
         <v>10</v>
       </c>
@@ -2072,7 +2076,11 @@
           <t>314-6CG23 VIPA CPU 314SC DPM</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
       <c r="E55" t="n">
         <v>7.5</v>
       </c>
@@ -2165,11 +2173,7 @@
           <t>972-ODPIO EasyConn 900 PB plug</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>85366990</t>
-        </is>
-      </c>
+      <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
         <v>10</v>
       </c>
@@ -2187,22 +2191,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>955-CO00MO00</t>
+          <t>031-1BB90</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>955-CO00MO00 - VIPASetCard 001 (VSC)</t>
+          <t>031-1BB90 - SM 031 - Analog input</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>85235100</t>
+          <t>85381010</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -2214,18 +2218,18 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>955-CO000MO00</t>
+          <t>SW110T1MA</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>955-CO000MO00 - VIPASetCard 001 (VSC)</t>
+          <t>SW110T1MA - OPC Server S7 TCP/IP License</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>85235100</t>
+          <t>49119990</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2233,195 +2237,6 @@
       </c>
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>955-CO00M00</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr"/>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>955-CO00M00 - VIPASetCard 001 (VSC)</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>85235100</t>
-        </is>
-      </c>
-      <c r="E61" t="n">
-        <v>10</v>
-      </c>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>315-4NE23</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr"/>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>315-4NE23 - VIPA CPU 315SN</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
-      <c r="E62" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>955-COO00MO00</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr"/>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>955-COO00MO00 - VIPASetCard 001 (VSC)</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>85235100</t>
-        </is>
-      </c>
-      <c r="E63" t="n">
-        <v>10</v>
-      </c>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>007-0AA00</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr"/>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>007-0AA00 - PM 007 - Power module</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>85369090</t>
-        </is>
-      </c>
-      <c r="E64" t="n">
-        <v>10</v>
-      </c>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>021-1BD40</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr"/>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>021-1BD40 - SM 021 - Digital input</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
-      <c r="E65" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>022-1BB90</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr"/>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>022-1BB90 - SM 022 - Digital output</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
-      <c r="E66" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>031-1BB90</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr"/>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>031-1BB90 - SM 031 - Analog input</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
-      <c r="E67" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>

</xml_diff>

<commit_message>
Fix native invoice PDF layout text extraction and part number normalization
</commit_message>
<xml_diff>
--- a/output/master_reviewed.xlsx
+++ b/output/master_reviewed.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +543,11 @@
           <t>032-1 CD70 SM 032 Analog output</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
       <c r="E4" t="n">
         <v>7.5</v>
       </c>
@@ -574,7 +578,11 @@
           <t>972-0DP30 EasyConn 00 PB plug</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>85366990</t>
+        </is>
+      </c>
       <c r="E5" t="n">
         <v>10</v>
       </c>
@@ -605,7 +613,11 @@
           <t>001-1 BAOO CM 001 Pot. distributor</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>85369090</t>
+        </is>
+      </c>
       <c r="E6" t="n">
         <v>10</v>
       </c>
@@ -636,7 +648,11 @@
           <t>001-1BAIO CM 001 pot. distributor</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>85369090</t>
+        </is>
+      </c>
       <c r="E7" t="n">
         <v>10</v>
       </c>
@@ -667,11 +683,7 @@
           <t>007-IABOO PM 007 Power module</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>85366990</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="n">
         <v>10</v>
       </c>
@@ -702,11 +714,7 @@
           <t>021-1 BFOO SM 021 Digital input</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
         <v>7.5</v>
       </c>
@@ -1150,7 +1158,11 @@
           <t>314-2AG23 VIPA CPU 314SB DPM</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
       <c r="E25" t="n">
         <v>7.5</v>
       </c>
@@ -1374,11 +1386,7 @@
           <t>031-1BD40 SM 031 Analog input</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>85381010</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="n">
         <v>7.5</v>
       </c>
@@ -1533,7 +1541,11 @@
           <t>032-1 BB40 SM 032 Analog output</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
       <c r="E38" t="n">
         <v>7.5</v>
       </c>
@@ -1719,11 +1731,7 @@
           <t>H41-71A41-0 smartPanel TP304-SM</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="n">
         <v>7.5</v>
       </c>
@@ -1754,11 +1762,7 @@
           <t>1-171-71 A 41-0 smartPanel TP307-SM</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="n">
         <v>7.5</v>
       </c>
@@ -1948,11 +1952,7 @@
           <t>001-1BA20 CM 001 pot. distributor</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>85366990</t>
-        </is>
-      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="n">
         <v>10</v>
       </c>
@@ -2076,11 +2076,7 @@
           <t>314-6CG23 VIPA CPU 314SC DPM</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
         <v>7.5</v>
       </c>
@@ -2173,7 +2169,11 @@
           <t>972-ODPIO EasyConn 900 PB plug</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>85366990</t>
+        </is>
+      </c>
       <c r="E58" t="n">
         <v>10</v>
       </c>
@@ -2191,22 +2191,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>031-1BB90</t>
+          <t>955-C000M00</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>031-1BB90 - SM 031 - Analog input</t>
+          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>85381010</t>
+          <t>85235100</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -2218,18 +2218,18 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SW110T1MA</t>
+          <t>955-C000M00</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>SW110T1MA - OPC Server S7 TCP/IP License</t>
+          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>49119990</t>
+          <t>85235100</t>
         </is>
       </c>
       <c r="E60" t="n">
@@ -2237,6 +2237,195 @@
       </c>
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>955-C000M00</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>85235100</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>10</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>315-4NE23</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>315-4NE23 -VIPA CPU 315SN</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>85371090</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>955-C000M00</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>85235100</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>10</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>007-0AA00</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>007-0AA00 - PM 007 - Power module</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>85369090</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>10</v>
+      </c>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>021-1BD40</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr"/>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>021-1 BD40 - SM 021 - Digital input</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>022-1BB90</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>022-1 B890 - SM 022 - Digital output</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>031-1BB90</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr"/>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>031-18B90 - SM 031 - Analog input</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>85381010</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
         <is>
           <t>NEW</t>
         </is>

</xml_diff>

<commit_message>
Update output workbooks with corrected PO numbers and add latest shipment files
</commit_message>
<xml_diff>
--- a/output/master_reviewed.xlsx
+++ b/output/master_reviewed.xlsx
@@ -1824,11 +1824,7 @@
           <t>015-CEFPROI CPU 015PN</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>85371090</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="n">
         <v>7.5</v>
       </c>
@@ -2191,13 +2187,13 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>955-C000M00</t>
+          <t>955-CO00MO00</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
-          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
+          <t>955-CO00MO00 - VIPASetCard 001 (VSC)</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2218,13 +2214,13 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>955-C000M00</t>
+          <t>955-CO000MO00</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
-          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
+          <t>955-CO000MO00 - VIPASetCard 001 (VSC)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2245,13 +2241,13 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>955-C000M00</t>
+          <t>955-CO00M00</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
-          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
+          <t>955-CO00M00 - VIPASetCard 001 (VSC)</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2278,7 +2274,7 @@
       <c r="B62" s="2" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
-          <t>315-4NE23 -VIPA CPU 315SN</t>
+          <t>315-4NE23 - VIPA CPU 315SN</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2299,13 +2295,13 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>955-C000M00</t>
+          <t>955-COO00MO00</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
-          <t>955-C000M00 - VIPASetCard 001 (VSC)</t>
+          <t>955-COO00MO00 - VIPASetCard 001 (VSC)</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2359,7 +2355,7 @@
       <c r="B65" s="2" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
-          <t>021-1 BD40 - SM 021 - Digital input</t>
+          <t>021-1BD40 - SM 021 - Digital input</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2386,7 +2382,7 @@
       <c r="B66" s="2" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
-          <t>022-1 B890 - SM 022 - Digital output</t>
+          <t>022-1BB90 - SM 022 - Digital output</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2413,7 +2409,7 @@
       <c r="B67" s="2" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
-          <t>031-18B90 - SM 031 - Analog input</t>
+          <t>031-1BB90 - SM 031 - Analog input</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">

</xml_diff>